<commit_message>
FIT: not shown anywhere a customer looks, kept everywhere it can come back
The keyword is not ready to stand behind yet, so the README bullet and the
template's `# MODULE id FIT member B/E target [GAP]` block are commented
out rather than deleted. The engine still reads FIT, so a sheet that
already uses it keeps running - this only stops us teaching it. One line
of the template's own prose said "A BASE or a FIT row wants the numbered
name"; it now says "A BASE row".

PLATE3D_TEMPLATE.xlsx regenerated and compared row by row against the old
one: 159 rows to 154, and the difference is exactly the note, the header,
the three blank rows under it, and that one sentence. Nothing else moved.

format unchanged · 2 books · 15 dimstyle constants · 24 keyword tables;
tutorial 62 checks pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnGhhpynbq7sNRTi2ok7Eu
</commit_message>
<xml_diff>
--- a/plate3d/PLATE3D_TEMPLATE.xlsx
+++ b/plate3d/PLATE3D_TEMPLATE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="199">
   <si>
     <t># PLATE3D  ·  blank input sheet</t>
   </si>
@@ -367,18 +367,6 @@
     <t>point</t>
   </si>
   <si>
-    <t>#   cut one end of a member to the face it runs into. B = start, E = end.</t>
-  </si>
-  <si>
-    <t>FIT</t>
-  </si>
-  <si>
-    <t>B / E</t>
-  </si>
-  <si>
-    <t>[GAP]</t>
-  </si>
-  <si>
     <t># 4.  ASSY  ·  modules, plates and bars into the world</t>
   </si>
   <si>
@@ -583,7 +571,7 @@
     <t>Name the same part as often as you use it - the engine numbers the repeats</t>
   </si>
   <si>
-    <t>itself, pl.stf twice becoming pl.stf_1 and pl.stf_2. A BASE or a FIT row</t>
+    <t>itself, pl.stf twice becoming pl.stf_1 and pl.stf_2. A BASE row</t>
   </si>
   <si>
     <t>wants the numbered name.</t>
@@ -1042,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R159"/>
+  <dimension ref="B1:R154"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -1769,383 +1757,384 @@
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="88" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B88" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C88" s="4" t="s">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B88" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B89" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B91" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C91" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D88" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="E88" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="F88" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G88" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="H88" s="4" t="s">
+      <c r="D91" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H91" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J91" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="K91" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="92" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B92" s="3" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B92" s="1" t="s">
+      <c r="C92" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D92" s="4" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B93" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B94" s="2" t="s">
+      <c r="E92" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F92" s="4" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B96" s="3" t="s">
+      <c r="G92" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C96" s="4" t="s">
+      <c r="H92" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="93" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B93" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C93" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D96" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="F96" s="4" t="s">
+      <c r="D93" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E93" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="G96" s="4" t="s">
+      <c r="F93" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="H96" s="4" t="s">
+      <c r="G93" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="I96" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="J96" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="K96" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="97" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B97" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C97" s="4" t="s">
+      <c r="H93" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="I93" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B94" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C94" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D97" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="E97" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F97" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="G97" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="H97" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="I97" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="98" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B98" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="E98" s="4" t="s">
+      <c r="D94" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E94" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="F94" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="G94" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="H94" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="J94" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="K94" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F98" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G98" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="H98" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="I98" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="99" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B99" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D99" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G99" s="4" t="s">
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B95" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="H99" s="4" t="s">
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="I99" s="4" t="s">
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B101" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="J99" s="4" t="s">
+    </row>
+    <row r="103" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B103" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="K99" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B100" s="2" t="s">
+      <c r="C103" s="4" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B105" s="1" t="s">
+      <c r="D103" s="4" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B106" s="2" t="s">
+      <c r="E103" s="4" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="108" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B108" s="3" t="s">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B104" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C108" s="4" t="s">
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B108" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D108" s="4" t="s">
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B111" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E108" s="4" t="s">
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B112" s="6"/>
+    </row>
+    <row r="113" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B113" s="6" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B109" s="2" t="s">
+      <c r="E113" s="7" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B113" s="5" t="s">
+    <row r="114" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B114" s="6"/>
+      <c r="E114" s="7" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B116" s="6" t="s">
+      <c r="F114" s="7" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G114" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="115" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B115" s="6"/>
+      <c r="E115" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F115" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="G115" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H115" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="116" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B116" s="6"/>
+      <c r="E116" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="F116" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="G116" s="7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="117" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B117" s="6"/>
-    </row>
-    <row r="118" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B118" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="E118" s="7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B119" s="6"/>
+      <c r="E117" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B118" s="6"/>
+    </row>
+    <row r="119" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B119" s="6" t="s">
+        <v>162</v>
+      </c>
       <c r="E119" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="F119" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="G119" s="7" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="120" spans="2:8" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="120" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B120" s="6"/>
       <c r="E120" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F120" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="G120" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="H120" s="7" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="6"/>
-      <c r="E121" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="F121" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="G121" s="7" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="122" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B122" s="6"/>
+      <c r="B122" s="6" t="s">
+        <v>165</v>
+      </c>
       <c r="E122" s="7" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="123" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B123" s="6"/>
+      <c r="E123" s="7" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="124" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B124" s="6" t="s">
-        <v>166</v>
-      </c>
+      <c r="B124" s="6"/>
       <c r="E124" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="125" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B125" s="6"/>
       <c r="E125" s="7" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="126" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B126" s="6"/>
-    </row>
-    <row r="127" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B127" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="E127" s="7" t="s">
+      <c r="E126" s="7" t="s">
         <v>170</v>
       </c>
     </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B127" s="6"/>
+    </row>
     <row r="128" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B128" s="6"/>
+      <c r="B128" s="6" t="s">
+        <v>171</v>
+      </c>
       <c r="E128" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="129" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B129" s="6"/>
       <c r="E129" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="130" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B130" s="6"/>
       <c r="E130" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="131" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B131" s="6"/>
       <c r="E131" s="7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="132" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B132" s="6"/>
-    </row>
-    <row r="133" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B133" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="E133" s="7" t="s">
+      <c r="E132" s="7" t="s">
         <v>176</v>
       </c>
     </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B133" s="6"/>
+    </row>
     <row r="134" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B134" s="6"/>
+      <c r="B134" s="6" t="s">
+        <v>177</v>
+      </c>
       <c r="E134" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="135" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B135" s="6"/>
       <c r="E135" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="136" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B136" s="6"/>
       <c r="E136" s="7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="137" spans="2:5" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="6"/>
-      <c r="E137" s="7" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B138" s="6"/>
-    </row>
-    <row r="139" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B139" s="6" t="s">
+    </row>
+    <row r="138" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B138" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E139" s="7" t="s">
+      <c r="E138" s="7" t="s">
         <v>182</v>
       </c>
     </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B139" s="6"/>
+    </row>
     <row r="140" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B140" s="6"/>
+      <c r="B140" s="6" t="s">
+        <v>183</v>
+      </c>
       <c r="E140" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="141" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B141" s="6"/>
       <c r="E141" s="7" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="142" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B142" s="6"/>
+      <c r="E142" s="7" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="143" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B143" s="6" t="s">
-        <v>185</v>
-      </c>
+      <c r="B143" s="6"/>
       <c r="E143" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="144" spans="2:2" x14ac:dyDescent="0.25">
@@ -2153,28 +2142,27 @@
     </row>
     <row r="145" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B145" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E145" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="146" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B146" s="6"/>
       <c r="E146" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="147" spans="2:5" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="6"/>
-      <c r="E147" s="7" t="s">
-        <v>190</v>
-      </c>
     </row>
     <row r="148" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B148" s="6"/>
+      <c r="B148" s="6" t="s">
+        <v>191</v>
+      </c>
       <c r="E148" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="149" spans="2:2" x14ac:dyDescent="0.25">
@@ -2182,16 +2170,16 @@
     </row>
     <row r="150" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B150" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E150" s="7" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="151" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B151" s="6"/>
       <c r="E151" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="152" spans="2:2" x14ac:dyDescent="0.25">
@@ -2199,44 +2187,16 @@
     </row>
     <row r="153" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B153" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E153" s="7" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="154" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B154" s="6"/>
-    </row>
-    <row r="155" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B155" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="E155" s="7" t="s">
+      <c r="E154" s="7" t="s">
         <v>198</v>
-      </c>
-    </row>
-    <row r="156" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B156" s="6"/>
-      <c r="E156" s="7" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B157" s="6"/>
-    </row>
-    <row r="158" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B158" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="E158" s="7" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="159" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B159" s="6"/>
-      <c r="E159" s="7" t="s">
-        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>